<commit_message>
fixed the issue suggeested by Prena on 6/7/2026
</commit_message>
<xml_diff>
--- a/pds_admin_Punjab_R/Backend/Backend/Tagging_Sheet_Pre.xlsx
+++ b/pds_admin_Punjab_R/Backend/Backend/Tagging_Sheet_Pre.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="265" uniqueCount="13">
   <si>
     <t>PC_ID</t>
   </si>
@@ -31,7 +31,28 @@
     <t>Values</t>
   </si>
   <si>
-    <t>stor</t>
+    <t>ajnala</t>
+  </si>
+  <si>
+    <t>ahmedgarh</t>
+  </si>
+  <si>
+    <t>majitha</t>
+  </si>
+  <si>
+    <t>abohar</t>
+  </si>
+  <si>
+    <t>adampur</t>
+  </si>
+  <si>
+    <t>rayya</t>
+  </si>
+  <si>
+    <t>chogawan</t>
+  </si>
+  <si>
+    <t>jandiala</t>
   </si>
 </sst>
 </file>
@@ -389,7 +410,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E84"/>
+  <dimension ref="A1:E131"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:5">
@@ -411,1413 +432,2212 @@
     </row>
     <row r="2" spans="1:5">
       <c r="A2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="B2" t="s">
         <v>5</v>
       </c>
       <c r="C2">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
       </c>
       <c r="E2">
-        <v>50000</v>
+        <v>160000</v>
       </c>
     </row>
     <row r="3" spans="1:5">
       <c r="A3">
-        <v>23</v>
+        <v>1</v>
       </c>
       <c r="B3" t="s">
         <v>5</v>
       </c>
       <c r="C3">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D3" t="s">
         <v>5</v>
       </c>
       <c r="E3">
-        <v>50000</v>
+        <v>132250</v>
       </c>
     </row>
     <row r="4" spans="1:5">
       <c r="A4">
-        <v>501</v>
+        <v>1</v>
       </c>
       <c r="B4" t="s">
         <v>5</v>
       </c>
       <c r="C4">
-        <v>396</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
         <v>5</v>
       </c>
       <c r="E4">
-        <v>90000</v>
+        <v>139400</v>
       </c>
     </row>
     <row r="5" spans="1:5">
       <c r="A5">
-        <v>501</v>
+        <v>3</v>
       </c>
       <c r="B5" t="s">
         <v>5</v>
       </c>
       <c r="C5">
-        <v>398</v>
+        <v>3</v>
       </c>
       <c r="D5" t="s">
         <v>5</v>
       </c>
       <c r="E5">
-        <v>60000</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="6" spans="1:5">
       <c r="A6">
-        <v>501</v>
+        <v>4</v>
       </c>
       <c r="B6" t="s">
         <v>5</v>
       </c>
       <c r="C6">
-        <v>399</v>
+        <v>2</v>
       </c>
       <c r="D6" t="s">
         <v>5</v>
       </c>
       <c r="E6">
-        <v>120000</v>
+        <v>17750</v>
       </c>
     </row>
     <row r="7" spans="1:5">
       <c r="A7">
-        <v>501</v>
+        <v>5</v>
       </c>
       <c r="B7" t="s">
         <v>5</v>
       </c>
       <c r="C7">
-        <v>400</v>
+        <v>23</v>
       </c>
       <c r="D7" t="s">
         <v>5</v>
       </c>
       <c r="E7">
-        <v>33610</v>
+        <v>12425</v>
       </c>
     </row>
     <row r="8" spans="1:5">
       <c r="A8">
-        <v>501</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
         <v>5</v>
       </c>
       <c r="C8">
-        <v>405</v>
+        <v>23</v>
       </c>
       <c r="D8" t="s">
         <v>5</v>
       </c>
       <c r="E8">
-        <v>150000</v>
+        <v>98175</v>
       </c>
     </row>
     <row r="9" spans="1:5">
       <c r="A9">
-        <v>501</v>
+        <v>1322</v>
       </c>
       <c r="B9" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C9">
-        <v>407</v>
+        <v>864</v>
       </c>
       <c r="D9" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E9">
-        <v>143264</v>
+        <v>197630</v>
       </c>
     </row>
     <row r="10" spans="1:5">
       <c r="A10">
-        <v>502</v>
+        <v>1322</v>
       </c>
       <c r="B10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C10">
-        <v>394</v>
+        <v>865</v>
       </c>
       <c r="D10" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E10">
-        <v>48247.5</v>
+        <v>16680</v>
       </c>
     </row>
     <row r="11" spans="1:5">
       <c r="A11">
-        <v>502</v>
+        <v>1322</v>
       </c>
       <c r="B11" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C11">
-        <v>397</v>
+        <v>866</v>
       </c>
       <c r="D11" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E11">
-        <v>23588</v>
+        <v>42630</v>
       </c>
     </row>
     <row r="12" spans="1:5">
       <c r="A12">
-        <v>503</v>
+        <v>1322</v>
       </c>
       <c r="B12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12">
-        <v>404</v>
+        <v>868</v>
       </c>
       <c r="D12" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E12">
-        <v>73860.5</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="13" spans="1:5">
       <c r="A13">
-        <v>505</v>
+        <v>1322</v>
       </c>
       <c r="B13" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C13">
-        <v>407</v>
+        <v>869</v>
       </c>
       <c r="D13" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E13">
-        <v>37309</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="14" spans="1:5">
       <c r="A14">
-        <v>506</v>
+        <v>1322</v>
       </c>
       <c r="B14" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C14">
-        <v>407</v>
+        <v>870</v>
       </c>
       <c r="D14" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E14">
-        <v>18025.5</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="15" spans="1:5">
       <c r="A15">
-        <v>507</v>
+        <v>1322</v>
       </c>
       <c r="B15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C15">
-        <v>394</v>
+        <v>871</v>
       </c>
       <c r="D15" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E15">
-        <v>16177.5</v>
+        <v>30720</v>
       </c>
     </row>
     <row r="16" spans="1:5">
       <c r="A16">
-        <v>507</v>
+        <v>1322</v>
       </c>
       <c r="B16" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C16">
-        <v>395</v>
+        <v>872</v>
       </c>
       <c r="D16" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E16">
-        <v>33588.5</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="17" spans="1:5">
       <c r="A17">
-        <v>508</v>
+        <v>1322</v>
       </c>
       <c r="B17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C17">
-        <v>403</v>
+        <v>873</v>
       </c>
       <c r="D17" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E17">
-        <v>13129</v>
+        <v>29640</v>
       </c>
     </row>
     <row r="18" spans="1:5">
       <c r="A18">
-        <v>508</v>
+        <v>1322</v>
       </c>
       <c r="B18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C18">
-        <v>407</v>
+        <v>877</v>
       </c>
       <c r="D18" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E18">
-        <v>28578.5</v>
+        <v>9950</v>
       </c>
     </row>
     <row r="19" spans="1:5">
       <c r="A19">
-        <v>509</v>
+        <v>1323</v>
       </c>
       <c r="B19" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C19">
-        <v>400</v>
+        <v>867</v>
       </c>
       <c r="D19" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E19">
-        <v>18038</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="20" spans="1:5">
       <c r="A20">
-        <v>510</v>
+        <v>1323</v>
       </c>
       <c r="B20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C20">
-        <v>407</v>
+        <v>875</v>
       </c>
       <c r="D20" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E20">
-        <v>44568.5</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="21" spans="1:5">
       <c r="A21">
-        <v>511</v>
+        <v>1323</v>
       </c>
       <c r="B21" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C21">
-        <v>397</v>
+        <v>876</v>
       </c>
       <c r="D21" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E21">
-        <v>25216</v>
+        <v>5000</v>
       </c>
     </row>
     <row r="22" spans="1:5">
       <c r="A22">
-        <v>512</v>
+        <v>1323</v>
       </c>
       <c r="B22" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C22">
-        <v>401</v>
+        <v>878</v>
       </c>
       <c r="D22" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E22">
-        <v>44802</v>
+        <v>20480</v>
       </c>
     </row>
     <row r="23" spans="1:5">
       <c r="A23">
-        <v>513</v>
+        <v>1323</v>
       </c>
       <c r="B23" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C23">
-        <v>407</v>
+        <v>879</v>
       </c>
       <c r="D23" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E23">
-        <v>30276.5</v>
+        <v>18000</v>
       </c>
     </row>
     <row r="24" spans="1:5">
       <c r="A24">
-        <v>514</v>
+        <v>1324</v>
       </c>
       <c r="B24" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C24">
-        <v>395</v>
+        <v>864</v>
       </c>
       <c r="D24" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E24">
-        <v>19961.5</v>
+        <v>41830</v>
       </c>
     </row>
     <row r="25" spans="1:5">
       <c r="A25">
-        <v>515</v>
+        <v>1325</v>
       </c>
       <c r="B25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C25">
-        <v>394</v>
+        <v>864</v>
       </c>
       <c r="D25" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E25">
-        <v>64381</v>
+        <v>55220</v>
       </c>
     </row>
     <row r="26" spans="1:5">
       <c r="A26">
-        <v>517</v>
+        <v>1326</v>
       </c>
       <c r="B26" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C26">
-        <v>400</v>
+        <v>866</v>
       </c>
       <c r="D26" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E26">
-        <v>39817.5</v>
+        <v>13140</v>
       </c>
     </row>
     <row r="27" spans="1:5">
       <c r="A27">
-        <v>518</v>
+        <v>1326</v>
       </c>
       <c r="B27" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C27">
-        <v>403</v>
+        <v>874</v>
       </c>
       <c r="D27" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E27">
-        <v>10375.5</v>
+        <v>28460</v>
       </c>
     </row>
     <row r="28" spans="1:5">
       <c r="A28">
-        <v>520</v>
+        <v>1326</v>
       </c>
       <c r="B28" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C28">
-        <v>407</v>
+        <v>879</v>
       </c>
       <c r="D28" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E28">
-        <v>100949.5</v>
+        <v>2480</v>
       </c>
     </row>
     <row r="29" spans="1:5">
       <c r="A29">
-        <v>521</v>
+        <v>1327</v>
       </c>
       <c r="B29" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C29">
-        <v>402</v>
+        <v>866</v>
       </c>
       <c r="D29" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E29">
-        <v>36622.5</v>
+        <v>59240</v>
       </c>
     </row>
     <row r="30" spans="1:5">
       <c r="A30">
-        <v>522</v>
+        <v>1328</v>
       </c>
       <c r="B30" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C30">
-        <v>404</v>
+        <v>866</v>
       </c>
       <c r="D30" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E30">
-        <v>11652.5</v>
+        <v>11670</v>
       </c>
     </row>
     <row r="31" spans="1:5">
       <c r="A31">
-        <v>522</v>
+        <v>1328</v>
       </c>
       <c r="B31" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C31">
-        <v>407</v>
+        <v>880</v>
       </c>
       <c r="D31" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E31">
-        <v>16592.5</v>
+        <v>15360</v>
       </c>
     </row>
     <row r="32" spans="1:5">
       <c r="A32">
-        <v>525</v>
+        <v>1329</v>
       </c>
       <c r="B32" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C32">
-        <v>407</v>
+        <v>877</v>
       </c>
       <c r="D32" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E32">
-        <v>21311</v>
+        <v>10530</v>
       </c>
     </row>
     <row r="33" spans="1:5">
       <c r="A33">
-        <v>526</v>
+        <v>1330</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C33">
-        <v>394</v>
+        <v>872</v>
       </c>
       <c r="D33" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E33">
-        <v>34094</v>
+        <v>29640</v>
       </c>
     </row>
     <row r="34" spans="1:5">
       <c r="A34">
-        <v>527</v>
+        <v>43</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C34">
-        <v>403</v>
+        <v>38</v>
       </c>
       <c r="D34" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E34">
-        <v>10795.5</v>
+        <v>35025</v>
       </c>
     </row>
     <row r="35" spans="1:5">
       <c r="A35">
-        <v>527</v>
+        <v>44</v>
       </c>
       <c r="B35" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C35">
-        <v>406</v>
+        <v>38</v>
       </c>
       <c r="D35" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E35">
-        <v>21605.5</v>
+        <v>52002</v>
       </c>
     </row>
     <row r="36" spans="1:5">
       <c r="A36">
-        <v>528</v>
+        <v>45</v>
       </c>
       <c r="B36" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C36">
-        <v>397</v>
+        <v>15</v>
       </c>
       <c r="D36" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E36">
-        <v>71196</v>
+        <v>137745</v>
       </c>
     </row>
     <row r="37" spans="1:5">
       <c r="A37">
-        <v>528</v>
+        <v>45</v>
       </c>
       <c r="B37" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C37">
-        <v>407</v>
+        <v>16</v>
       </c>
       <c r="D37" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E37">
-        <v>2489</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="38" spans="1:5">
       <c r="A38">
-        <v>529</v>
+        <v>45</v>
       </c>
       <c r="B38" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C38">
-        <v>407</v>
+        <v>38</v>
       </c>
       <c r="D38" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E38">
-        <v>34208</v>
+        <v>12973</v>
       </c>
     </row>
     <row r="39" spans="1:5">
       <c r="A39">
-        <v>531</v>
+        <v>45</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C39">
-        <v>400</v>
+        <v>39</v>
       </c>
       <c r="D39" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E39">
-        <v>54819.5</v>
+        <v>50000</v>
       </c>
     </row>
     <row r="40" spans="1:5">
       <c r="A40">
-        <v>532</v>
+        <v>46</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C40">
-        <v>407</v>
+        <v>15</v>
       </c>
       <c r="D40" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E40">
-        <v>37768</v>
+        <v>42255</v>
       </c>
     </row>
     <row r="41" spans="1:5">
       <c r="A41">
-        <v>533</v>
+        <v>46</v>
       </c>
       <c r="B41" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C41">
-        <v>407</v>
+        <v>45</v>
       </c>
       <c r="D41" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E41">
-        <v>29874.5</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="42" spans="1:5">
       <c r="A42">
-        <v>534</v>
+        <v>46</v>
       </c>
       <c r="B42" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C42">
-        <v>407</v>
+        <v>46</v>
       </c>
       <c r="D42" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E42">
-        <v>56983.5</v>
+        <v>25000</v>
       </c>
     </row>
     <row r="43" spans="1:5">
       <c r="A43">
-        <v>535</v>
+        <v>501</v>
       </c>
       <c r="B43" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C43">
-        <v>407</v>
+        <v>396</v>
       </c>
       <c r="D43" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E43">
-        <v>23195.5</v>
+        <v>90000</v>
       </c>
     </row>
     <row r="44" spans="1:5">
       <c r="A44">
-        <v>538</v>
+        <v>501</v>
       </c>
       <c r="B44" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C44">
-        <v>407</v>
+        <v>398</v>
       </c>
       <c r="D44" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E44">
-        <v>57368</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="45" spans="1:5">
       <c r="A45">
-        <v>540</v>
+        <v>501</v>
       </c>
       <c r="B45" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C45">
-        <v>404</v>
+        <v>399</v>
       </c>
       <c r="D45" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E45">
-        <v>2487</v>
+        <v>120000</v>
       </c>
     </row>
     <row r="46" spans="1:5">
       <c r="A46">
-        <v>541</v>
+        <v>501</v>
       </c>
       <c r="B46" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C46">
         <v>400</v>
       </c>
       <c r="D46" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E46">
-        <v>29195</v>
+        <v>145397</v>
       </c>
     </row>
     <row r="47" spans="1:5">
       <c r="A47">
-        <v>542</v>
+        <v>501</v>
       </c>
       <c r="B47" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C47">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="D47" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E47">
-        <v>26795</v>
+        <v>31477</v>
       </c>
     </row>
     <row r="48" spans="1:5">
       <c r="A48">
-        <v>543</v>
+        <v>501</v>
       </c>
       <c r="B48" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C48">
-        <v>400</v>
+        <v>405</v>
       </c>
       <c r="D48" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E48">
-        <v>7950</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="49" spans="1:5">
       <c r="A49">
-        <v>545</v>
+        <v>502</v>
       </c>
       <c r="B49" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C49">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="D49" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E49">
-        <v>5500</v>
+        <v>71835.5</v>
       </c>
     </row>
     <row r="50" spans="1:5">
       <c r="A50">
-        <v>546</v>
+        <v>503</v>
       </c>
       <c r="B50" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C50">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="D50" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E50">
-        <v>12630.5</v>
+        <v>73538.5</v>
       </c>
     </row>
     <row r="51" spans="1:5">
       <c r="A51">
-        <v>547</v>
+        <v>503</v>
       </c>
       <c r="B51" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C51">
         <v>407</v>
       </c>
       <c r="D51" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E51">
-        <v>13803</v>
+        <v>322</v>
       </c>
     </row>
     <row r="52" spans="1:5">
       <c r="A52">
-        <v>548</v>
+        <v>505</v>
       </c>
       <c r="B52" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C52">
         <v>407</v>
       </c>
       <c r="D52" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E52">
-        <v>9145</v>
+        <v>37309</v>
       </c>
     </row>
     <row r="53" spans="1:5">
       <c r="A53">
-        <v>549</v>
+        <v>506</v>
       </c>
       <c r="B53" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C53">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="D53" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E53">
-        <v>17622.5</v>
+        <v>2823</v>
       </c>
     </row>
     <row r="54" spans="1:5">
       <c r="A54">
-        <v>550</v>
+        <v>506</v>
       </c>
       <c r="B54" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C54">
-        <v>400</v>
+        <v>406</v>
       </c>
       <c r="D54" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E54">
-        <v>2347.5</v>
+        <v>15202.5</v>
       </c>
     </row>
     <row r="55" spans="1:5">
       <c r="A55">
-        <v>550</v>
+        <v>507</v>
       </c>
       <c r="B55" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C55">
-        <v>402</v>
+        <v>395</v>
       </c>
       <c r="D55" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E55">
-        <v>40337.5</v>
+        <v>49766</v>
       </c>
     </row>
     <row r="56" spans="1:5">
       <c r="A56">
-        <v>551</v>
+        <v>508</v>
       </c>
       <c r="B56" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C56">
-        <v>401</v>
+        <v>406</v>
       </c>
       <c r="D56" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E56">
-        <v>56502.5</v>
+        <v>41707.5</v>
       </c>
     </row>
     <row r="57" spans="1:5">
       <c r="A57">
-        <v>552</v>
+        <v>509</v>
       </c>
       <c r="B57" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C57">
-        <v>401</v>
+        <v>400</v>
       </c>
       <c r="D57" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E57">
-        <v>43110</v>
+        <v>18038</v>
       </c>
     </row>
     <row r="58" spans="1:5">
       <c r="A58">
-        <v>560</v>
+        <v>510</v>
       </c>
       <c r="B58" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C58">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="D58" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E58">
-        <v>128218</v>
+        <v>44568.5</v>
       </c>
     </row>
     <row r="59" spans="1:5">
       <c r="A59">
-        <v>565</v>
+        <v>511</v>
       </c>
       <c r="B59" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C59">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="D59" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E59">
-        <v>62709.5</v>
+        <v>25216</v>
       </c>
     </row>
     <row r="60" spans="1:5">
       <c r="A60">
-        <v>612</v>
+        <v>512</v>
       </c>
       <c r="B60" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C60">
         <v>401</v>
       </c>
       <c r="D60" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E60">
-        <v>47189.5</v>
+        <v>44802</v>
       </c>
     </row>
     <row r="61" spans="1:5">
       <c r="A61">
-        <v>1046</v>
+        <v>513</v>
       </c>
       <c r="B61" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C61">
-        <v>625</v>
+        <v>407</v>
       </c>
       <c r="D61" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E61">
-        <v>21500</v>
+        <v>30276.5</v>
       </c>
     </row>
     <row r="62" spans="1:5">
       <c r="A62">
-        <v>1577</v>
+        <v>514</v>
       </c>
       <c r="B62" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C62">
-        <v>866</v>
+        <v>404</v>
       </c>
       <c r="D62" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E62">
-        <v>88594</v>
+        <v>19961.5</v>
       </c>
     </row>
     <row r="63" spans="1:5">
       <c r="A63">
-        <v>1577</v>
+        <v>515</v>
       </c>
       <c r="B63" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C63">
-        <v>870</v>
+        <v>397</v>
       </c>
       <c r="D63" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E63">
-        <v>10000</v>
+        <v>9709</v>
       </c>
     </row>
     <row r="64" spans="1:5">
       <c r="A64">
-        <v>1577</v>
+        <v>515</v>
       </c>
       <c r="B64" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C64">
-        <v>875</v>
+        <v>407</v>
       </c>
       <c r="D64" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E64">
-        <v>5000</v>
+        <v>54672</v>
       </c>
     </row>
     <row r="65" spans="1:5">
       <c r="A65">
-        <v>1577</v>
+        <v>516</v>
       </c>
       <c r="B65" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C65">
-        <v>876</v>
+        <v>401</v>
       </c>
       <c r="D65" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E65">
-        <v>5000</v>
+        <v>13755.5</v>
       </c>
     </row>
     <row r="66" spans="1:5">
       <c r="A66">
-        <v>1597</v>
+        <v>516</v>
       </c>
       <c r="B66" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C66">
-        <v>866</v>
+        <v>406</v>
       </c>
       <c r="D66" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E66">
-        <v>38086</v>
+        <v>6714.5</v>
       </c>
     </row>
     <row r="67" spans="1:5">
       <c r="A67">
-        <v>1597</v>
+        <v>517</v>
       </c>
       <c r="B67" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C67">
-        <v>872</v>
+        <v>400</v>
       </c>
       <c r="D67" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E67">
-        <v>30720</v>
+        <v>39817.5</v>
       </c>
     </row>
     <row r="68" spans="1:5">
       <c r="A68">
-        <v>1597</v>
+        <v>518</v>
       </c>
       <c r="B68" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C68">
-        <v>877</v>
+        <v>406</v>
       </c>
       <c r="D68" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E68">
-        <v>5127</v>
+        <v>10375.5</v>
       </c>
     </row>
     <row r="69" spans="1:5">
       <c r="A69">
-        <v>1607</v>
+        <v>520</v>
       </c>
       <c r="B69" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C69">
-        <v>864</v>
+        <v>400</v>
       </c>
       <c r="D69" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E69">
-        <v>294680</v>
+        <v>72343</v>
       </c>
     </row>
     <row r="70" spans="1:5">
       <c r="A70">
-        <v>1607</v>
+        <v>520</v>
       </c>
       <c r="B70" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C70">
-        <v>865</v>
+        <v>407</v>
       </c>
       <c r="D70" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E70">
-        <v>16680</v>
+        <v>28606.5</v>
       </c>
     </row>
     <row r="71" spans="1:5">
       <c r="A71">
-        <v>1607</v>
+        <v>521</v>
       </c>
       <c r="B71" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C71">
-        <v>867</v>
+        <v>401</v>
       </c>
       <c r="D71" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E71">
-        <v>10000</v>
+        <v>2347.5</v>
       </c>
     </row>
     <row r="72" spans="1:5">
       <c r="A72">
-        <v>1607</v>
+        <v>521</v>
       </c>
       <c r="B72" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C72">
-        <v>868</v>
+        <v>402</v>
       </c>
       <c r="D72" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E72">
-        <v>10000</v>
+        <v>34275</v>
       </c>
     </row>
     <row r="73" spans="1:5">
       <c r="A73">
-        <v>1607</v>
+        <v>522</v>
       </c>
       <c r="B73" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C73">
-        <v>869</v>
+        <v>407</v>
       </c>
       <c r="D73" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E73">
-        <v>10000</v>
+        <v>28245</v>
       </c>
     </row>
     <row r="74" spans="1:5">
       <c r="A74">
-        <v>1607</v>
+        <v>523</v>
       </c>
       <c r="B74" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C74">
-        <v>871</v>
+        <v>407</v>
       </c>
       <c r="D74" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E74">
-        <v>30720</v>
+        <v>12854</v>
       </c>
     </row>
     <row r="75" spans="1:5">
       <c r="A75">
-        <v>1607</v>
+        <v>524</v>
       </c>
       <c r="B75" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C75">
-        <v>873</v>
+        <v>397</v>
       </c>
       <c r="D75" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E75">
-        <v>29640</v>
+        <v>74081</v>
       </c>
     </row>
     <row r="76" spans="1:5">
       <c r="A76">
-        <v>1607</v>
+        <v>525</v>
       </c>
       <c r="B76" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C76">
-        <v>874</v>
+        <v>407</v>
       </c>
       <c r="D76" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E76">
-        <v>28460</v>
+        <v>21311</v>
       </c>
     </row>
     <row r="77" spans="1:5">
       <c r="A77">
-        <v>1607</v>
+        <v>526</v>
       </c>
       <c r="B77" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C77">
-        <v>877</v>
+        <v>394</v>
       </c>
       <c r="D77" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E77">
-        <v>15353</v>
+        <v>30310</v>
       </c>
     </row>
     <row r="78" spans="1:5">
       <c r="A78">
-        <v>1607</v>
+        <v>526</v>
       </c>
       <c r="B78" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C78">
-        <v>878</v>
+        <v>395</v>
       </c>
       <c r="D78" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E78">
-        <v>20480</v>
+        <v>3784</v>
       </c>
     </row>
     <row r="79" spans="1:5">
       <c r="A79">
-        <v>1607</v>
+        <v>527</v>
       </c>
       <c r="B79" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C79">
-        <v>879</v>
+        <v>401</v>
       </c>
       <c r="D79" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E79">
-        <v>20480</v>
+        <v>32401</v>
       </c>
     </row>
     <row r="80" spans="1:5">
       <c r="A80">
-        <v>1607</v>
+        <v>528</v>
       </c>
       <c r="B80" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C80">
-        <v>880</v>
+        <v>407</v>
       </c>
       <c r="D80" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E80">
-        <v>15360</v>
+        <v>73685</v>
       </c>
     </row>
     <row r="81" spans="1:5">
       <c r="A81">
-        <v>1660</v>
+        <v>529</v>
       </c>
       <c r="B81" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C81">
-        <v>401</v>
+        <v>407</v>
       </c>
       <c r="D81" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E81">
-        <v>1314.5</v>
+        <v>34208</v>
       </c>
     </row>
     <row r="82" spans="1:5">
       <c r="A82">
-        <v>1660</v>
+        <v>530</v>
       </c>
       <c r="B82" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C82">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="D82" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E82">
-        <v>52394.5</v>
+        <v>17701</v>
       </c>
     </row>
     <row r="83" spans="1:5">
       <c r="A83">
-        <v>2153</v>
+        <v>531</v>
       </c>
       <c r="B83" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C83">
-        <v>2</v>
+        <v>400</v>
       </c>
       <c r="D83" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="E83">
-        <v>150000</v>
+        <v>54819.5</v>
       </c>
     </row>
     <row r="84" spans="1:5">
       <c r="A84">
-        <v>2153</v>
+        <v>532</v>
       </c>
       <c r="B84" t="s">
+        <v>8</v>
+      </c>
+      <c r="C84">
+        <v>407</v>
+      </c>
+      <c r="D84" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84">
+        <v>37768</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5">
+      <c r="A85">
+        <v>533</v>
+      </c>
+      <c r="B85" t="s">
+        <v>8</v>
+      </c>
+      <c r="C85">
+        <v>407</v>
+      </c>
+      <c r="D85" t="s">
+        <v>8</v>
+      </c>
+      <c r="E85">
+        <v>29874.5</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5">
+      <c r="A86">
+        <v>534</v>
+      </c>
+      <c r="B86" t="s">
+        <v>8</v>
+      </c>
+      <c r="C86">
+        <v>407</v>
+      </c>
+      <c r="D86" t="s">
+        <v>8</v>
+      </c>
+      <c r="E86">
+        <v>56983.5</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5">
+      <c r="A87">
+        <v>535</v>
+      </c>
+      <c r="B87" t="s">
+        <v>8</v>
+      </c>
+      <c r="C87">
+        <v>407</v>
+      </c>
+      <c r="D87" t="s">
+        <v>8</v>
+      </c>
+      <c r="E87">
+        <v>23195.5</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5">
+      <c r="A88">
+        <v>536</v>
+      </c>
+      <c r="B88" t="s">
+        <v>8</v>
+      </c>
+      <c r="C88">
+        <v>394</v>
+      </c>
+      <c r="D88" t="s">
+        <v>8</v>
+      </c>
+      <c r="E88">
+        <v>71340</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5">
+      <c r="A89">
+        <v>536</v>
+      </c>
+      <c r="B89" t="s">
+        <v>8</v>
+      </c>
+      <c r="C89">
+        <v>397</v>
+      </c>
+      <c r="D89" t="s">
+        <v>8</v>
+      </c>
+      <c r="E89">
+        <v>36210</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5">
+      <c r="A90">
+        <v>537</v>
+      </c>
+      <c r="B90" t="s">
+        <v>8</v>
+      </c>
+      <c r="C90">
+        <v>394</v>
+      </c>
+      <c r="D90" t="s">
+        <v>8</v>
+      </c>
+      <c r="E90">
+        <v>43549</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5">
+      <c r="A91">
+        <v>538</v>
+      </c>
+      <c r="B91" t="s">
+        <v>8</v>
+      </c>
+      <c r="C91">
+        <v>407</v>
+      </c>
+      <c r="D91" t="s">
+        <v>8</v>
+      </c>
+      <c r="E91">
+        <v>57368</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5">
+      <c r="A92">
+        <v>540</v>
+      </c>
+      <c r="B92" t="s">
+        <v>8</v>
+      </c>
+      <c r="C92">
+        <v>407</v>
+      </c>
+      <c r="D92" t="s">
+        <v>8</v>
+      </c>
+      <c r="E92">
+        <v>2487</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5">
+      <c r="A93">
+        <v>541</v>
+      </c>
+      <c r="B93" t="s">
+        <v>8</v>
+      </c>
+      <c r="C93">
+        <v>400</v>
+      </c>
+      <c r="D93" t="s">
+        <v>8</v>
+      </c>
+      <c r="E93">
+        <v>29195</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5">
+      <c r="A94">
+        <v>542</v>
+      </c>
+      <c r="B94" t="s">
+        <v>8</v>
+      </c>
+      <c r="C94">
+        <v>400</v>
+      </c>
+      <c r="D94" t="s">
+        <v>8</v>
+      </c>
+      <c r="E94">
+        <v>26795</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5">
+      <c r="A95">
+        <v>543</v>
+      </c>
+      <c r="B95" t="s">
+        <v>8</v>
+      </c>
+      <c r="C95">
+        <v>400</v>
+      </c>
+      <c r="D95" t="s">
+        <v>8</v>
+      </c>
+      <c r="E95">
+        <v>7950</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5">
+      <c r="A96">
+        <v>545</v>
+      </c>
+      <c r="B96" t="s">
+        <v>8</v>
+      </c>
+      <c r="C96">
+        <v>407</v>
+      </c>
+      <c r="D96" t="s">
+        <v>8</v>
+      </c>
+      <c r="E96">
+        <v>5500</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5">
+      <c r="A97">
+        <v>546</v>
+      </c>
+      <c r="B97" t="s">
+        <v>8</v>
+      </c>
+      <c r="C97">
+        <v>407</v>
+      </c>
+      <c r="D97" t="s">
+        <v>8</v>
+      </c>
+      <c r="E97">
+        <v>12630.5</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5">
+      <c r="A98">
+        <v>547</v>
+      </c>
+      <c r="B98" t="s">
+        <v>8</v>
+      </c>
+      <c r="C98">
+        <v>407</v>
+      </c>
+      <c r="D98" t="s">
+        <v>8</v>
+      </c>
+      <c r="E98">
+        <v>13803</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5">
+      <c r="A99">
+        <v>548</v>
+      </c>
+      <c r="B99" t="s">
+        <v>8</v>
+      </c>
+      <c r="C99">
+        <v>400</v>
+      </c>
+      <c r="D99" t="s">
+        <v>8</v>
+      </c>
+      <c r="E99">
+        <v>9145</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5">
+      <c r="A100">
+        <v>549</v>
+      </c>
+      <c r="B100" t="s">
+        <v>8</v>
+      </c>
+      <c r="C100">
+        <v>401</v>
+      </c>
+      <c r="D100" t="s">
+        <v>8</v>
+      </c>
+      <c r="E100">
+        <v>17622.5</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5">
+      <c r="A101">
+        <v>550</v>
+      </c>
+      <c r="B101" t="s">
+        <v>8</v>
+      </c>
+      <c r="C101">
+        <v>402</v>
+      </c>
+      <c r="D101" t="s">
+        <v>8</v>
+      </c>
+      <c r="E101">
+        <v>42685</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5">
+      <c r="A102">
+        <v>551</v>
+      </c>
+      <c r="B102" t="s">
+        <v>8</v>
+      </c>
+      <c r="C102">
+        <v>401</v>
+      </c>
+      <c r="D102" t="s">
+        <v>8</v>
+      </c>
+      <c r="E102">
+        <v>56502.5</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5">
+      <c r="A103">
+        <v>552</v>
+      </c>
+      <c r="B103" t="s">
+        <v>8</v>
+      </c>
+      <c r="C103">
+        <v>401</v>
+      </c>
+      <c r="D103" t="s">
+        <v>8</v>
+      </c>
+      <c r="E103">
+        <v>43110</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5">
+      <c r="A104">
+        <v>1046</v>
+      </c>
+      <c r="B104" t="s">
+        <v>9</v>
+      </c>
+      <c r="C104">
+        <v>625</v>
+      </c>
+      <c r="D104" t="s">
+        <v>9</v>
+      </c>
+      <c r="E104">
+        <v>21500</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5">
+      <c r="A105">
+        <v>54</v>
+      </c>
+      <c r="B105" t="s">
+        <v>10</v>
+      </c>
+      <c r="C105">
+        <v>21</v>
+      </c>
+      <c r="D105" t="s">
+        <v>10</v>
+      </c>
+      <c r="E105">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5">
+      <c r="A106">
+        <v>54</v>
+      </c>
+      <c r="B106" t="s">
+        <v>10</v>
+      </c>
+      <c r="C106">
+        <v>29</v>
+      </c>
+      <c r="D106" t="s">
+        <v>10</v>
+      </c>
+      <c r="E106">
+        <v>31832.5</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5">
+      <c r="A107">
+        <v>54</v>
+      </c>
+      <c r="B107" t="s">
+        <v>10</v>
+      </c>
+      <c r="C107">
+        <v>37</v>
+      </c>
+      <c r="D107" t="s">
+        <v>10</v>
+      </c>
+      <c r="E107">
+        <v>792</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5">
+      <c r="A108">
+        <v>54</v>
+      </c>
+      <c r="B108" t="s">
+        <v>10</v>
+      </c>
+      <c r="C108">
+        <v>44</v>
+      </c>
+      <c r="D108" t="s">
+        <v>10</v>
+      </c>
+      <c r="E108">
+        <v>12000</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5">
+      <c r="A109">
+        <v>55</v>
+      </c>
+      <c r="B109" t="s">
+        <v>10</v>
+      </c>
+      <c r="C109">
+        <v>29</v>
+      </c>
+      <c r="D109" t="s">
+        <v>10</v>
+      </c>
+      <c r="E109">
+        <v>17174.5</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5">
+      <c r="A110">
+        <v>56</v>
+      </c>
+      <c r="B110" t="s">
+        <v>10</v>
+      </c>
+      <c r="C110">
+        <v>29</v>
+      </c>
+      <c r="D110" t="s">
+        <v>10</v>
+      </c>
+      <c r="E110">
+        <v>25993</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5">
+      <c r="A111">
+        <v>57</v>
+      </c>
+      <c r="B111" t="s">
+        <v>10</v>
+      </c>
+      <c r="C111">
+        <v>19</v>
+      </c>
+      <c r="D111" t="s">
+        <v>10</v>
+      </c>
+      <c r="E111">
+        <v>190000</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5">
+      <c r="A112">
+        <v>57</v>
+      </c>
+      <c r="B112" t="s">
+        <v>10</v>
+      </c>
+      <c r="C112">
+        <v>20</v>
+      </c>
+      <c r="D112" t="s">
+        <v>10</v>
+      </c>
+      <c r="E112">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5">
+      <c r="A113">
+        <v>57</v>
+      </c>
+      <c r="B113" t="s">
+        <v>10</v>
+      </c>
+      <c r="C113">
+        <v>27</v>
+      </c>
+      <c r="D113" t="s">
+        <v>10</v>
+      </c>
+      <c r="E113">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5">
+      <c r="A114">
+        <v>57</v>
+      </c>
+      <c r="B114" t="s">
+        <v>10</v>
+      </c>
+      <c r="C114">
+        <v>28</v>
+      </c>
+      <c r="D114" t="s">
+        <v>10</v>
+      </c>
+      <c r="E114">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5">
+      <c r="A115">
+        <v>57</v>
+      </c>
+      <c r="B115" t="s">
+        <v>10</v>
+      </c>
+      <c r="C115">
+        <v>36</v>
+      </c>
+      <c r="D115" t="s">
+        <v>10</v>
+      </c>
+      <c r="E115">
+        <v>17870</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5">
+      <c r="A116">
+        <v>57</v>
+      </c>
+      <c r="B116" t="s">
+        <v>10</v>
+      </c>
+      <c r="C116">
+        <v>37</v>
+      </c>
+      <c r="D116" t="s">
+        <v>10</v>
+      </c>
+      <c r="E116">
+        <v>38457</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5">
+      <c r="A117">
+        <v>57</v>
+      </c>
+      <c r="B117" t="s">
+        <v>10</v>
+      </c>
+      <c r="C117">
+        <v>43</v>
+      </c>
+      <c r="D117" t="s">
+        <v>10</v>
+      </c>
+      <c r="E117">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5">
+      <c r="A118">
+        <v>58</v>
+      </c>
+      <c r="B118" t="s">
+        <v>10</v>
+      </c>
+      <c r="C118">
+        <v>17</v>
+      </c>
+      <c r="D118" t="s">
+        <v>10</v>
+      </c>
+      <c r="E118">
+        <v>17500</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5">
+      <c r="A119">
+        <v>58</v>
+      </c>
+      <c r="B119" t="s">
+        <v>10</v>
+      </c>
+      <c r="C119">
+        <v>18</v>
+      </c>
+      <c r="D119" t="s">
+        <v>10</v>
+      </c>
+      <c r="E119">
+        <v>17500</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5">
+      <c r="A120">
+        <v>58</v>
+      </c>
+      <c r="B120" t="s">
+        <v>10</v>
+      </c>
+      <c r="C120">
+        <v>35</v>
+      </c>
+      <c r="D120" t="s">
+        <v>10</v>
+      </c>
+      <c r="E120">
+        <v>7070</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5">
+      <c r="A121">
+        <v>58</v>
+      </c>
+      <c r="B121" t="s">
+        <v>10</v>
+      </c>
+      <c r="C121">
+        <v>37</v>
+      </c>
+      <c r="D121" t="s">
+        <v>10</v>
+      </c>
+      <c r="E121">
+        <v>90831</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5">
+      <c r="A122">
+        <v>23</v>
+      </c>
+      <c r="B122" t="s">
+        <v>11</v>
+      </c>
+      <c r="C122">
         <v>5</v>
       </c>
-      <c r="C84">
-        <v>4</v>
-      </c>
-      <c r="D84" t="s">
-        <v>5</v>
-      </c>
-      <c r="E84">
-        <v>150000</v>
+      <c r="D122" t="s">
+        <v>11</v>
+      </c>
+      <c r="E122">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5">
+      <c r="A123">
+        <v>24</v>
+      </c>
+      <c r="B123" t="s">
+        <v>11</v>
+      </c>
+      <c r="C123">
+        <v>11</v>
+      </c>
+      <c r="D123" t="s">
+        <v>11</v>
+      </c>
+      <c r="E123">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5">
+      <c r="A124">
+        <v>24</v>
+      </c>
+      <c r="B124" t="s">
+        <v>11</v>
+      </c>
+      <c r="C124">
+        <v>12</v>
+      </c>
+      <c r="D124" t="s">
+        <v>11</v>
+      </c>
+      <c r="E124">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5">
+      <c r="A125">
+        <v>36</v>
+      </c>
+      <c r="B125" t="s">
+        <v>12</v>
+      </c>
+      <c r="C125">
+        <v>13</v>
+      </c>
+      <c r="D125" t="s">
+        <v>12</v>
+      </c>
+      <c r="E125">
+        <v>5511</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5">
+      <c r="A126">
+        <v>36</v>
+      </c>
+      <c r="B126" t="s">
+        <v>12</v>
+      </c>
+      <c r="C126">
+        <v>14</v>
+      </c>
+      <c r="D126" t="s">
+        <v>12</v>
+      </c>
+      <c r="E126">
+        <v>70000</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5">
+      <c r="A127">
+        <v>36</v>
+      </c>
+      <c r="B127" t="s">
+        <v>12</v>
+      </c>
+      <c r="C127">
+        <v>30</v>
+      </c>
+      <c r="D127" t="s">
+        <v>12</v>
+      </c>
+      <c r="E127">
+        <v>25000</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5">
+      <c r="A128">
+        <v>36</v>
+      </c>
+      <c r="B128" t="s">
+        <v>12</v>
+      </c>
+      <c r="C128">
+        <v>31</v>
+      </c>
+      <c r="D128" t="s">
+        <v>12</v>
+      </c>
+      <c r="E128">
+        <v>10500</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5">
+      <c r="A129">
+        <v>36</v>
+      </c>
+      <c r="B129" t="s">
+        <v>12</v>
+      </c>
+      <c r="C129">
+        <v>34</v>
+      </c>
+      <c r="D129" t="s">
+        <v>12</v>
+      </c>
+      <c r="E129">
+        <v>5100</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5">
+      <c r="A130">
+        <v>38</v>
+      </c>
+      <c r="B130" t="s">
+        <v>12</v>
+      </c>
+      <c r="C130">
+        <v>13</v>
+      </c>
+      <c r="D130" t="s">
+        <v>12</v>
+      </c>
+      <c r="E130">
+        <v>88347</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5">
+      <c r="A131">
+        <v>40</v>
+      </c>
+      <c r="B131" t="s">
+        <v>12</v>
+      </c>
+      <c r="C131">
+        <v>13</v>
+      </c>
+      <c r="D131" t="s">
+        <v>12</v>
+      </c>
+      <c r="E131">
+        <v>11142</v>
       </c>
     </row>
   </sheetData>

</xml_diff>